<commit_message>
-Correcting some documentaion issues
</commit_message>
<xml_diff>
--- a/H0FR71/Released/BOM/H0FR71.xlsx
+++ b/H0FR71/Released/BOM/H0FR71.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HEXABITZ\Modules\Hardware\Modules Hardware Design\H0FR71\Final\H0FR71\Released\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HEXABITZ\Modules\Hardware\Modules Hardware Design\H0FR71\H0FR71\Released\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEFFF180-885C-4155-B193-EE462B97C72A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1457798-D0B8-4DA3-9EC6-012451C40E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="H21R00" sheetId="1" r:id="rId1"/>
+    <sheet name="H0FR71" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -590,7 +590,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -604,9 +604,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -617,7 +614,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
@@ -677,6 +673,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1054,525 +1068,525 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:G29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="70.5703125" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="84" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="53.77734375" style="32" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.5546875" style="32" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" customWidth="1"/>
     <col min="7" max="7" width="49" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="9" t="s">
+    <row r="2" spans="1:7" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="A2" s="6"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="14" t="s">
+      <c r="D2" s="7"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="B3" s="30"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="12"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="E3" s="30"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="34" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="24">
+      <c r="D4" s="22">
         <v>1</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="34" t="s">
         <v>71</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="23">
         <v>44772</v>
       </c>
-      <c r="E5" s="26"/>
-      <c r="F5" s="27"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="34" t="s">
         <v>114</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="30"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="28"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="31" t="s">
         <v>2</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="21">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+    <row r="11" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="16">
         <v>7</v>
       </c>
-      <c r="G15" s="21"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="G15" s="19"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+    <row r="18" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="16">
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
+    <row r="24" spans="1:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="16" t="s">
+      <c r="E24" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+    <row r="25" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="16">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="F27" s="18">
+      <c r="F27" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="F28" s="18">
+      <c r="F28" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="16">
         <v>1</v>
       </c>
     </row>

</xml_diff>